<commit_message>
Added new sections to the admin pannel, location and world gems along with classes and races
</commit_message>
<xml_diff>
--- a/resources/data-imports/Location Templates/location_templates.xlsx
+++ b/resources/data-imports/Location Templates/location_templates.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="2507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="2187">
   <si>
     <t>name</t>
   </si>
@@ -5420,390 +5420,6 @@
     <t>Gold Mine Waystation Pier keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
   </si>
   <si>
-    <t>Lords Stronghold Ash-Bent Hamlet</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Ash-Bent Hamlet from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Federation Scarred Road</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Federation Scarred Road from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Starving Lantern Camp</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Starving Lantern Camp from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Drowned Merchant Post</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Drowned Merchant Post from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Broken Watch House</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Broken Watch House from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Memory-Warped Shrine</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Memory-Warped Shrine from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Famished Orchard</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Famished Orchard from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Grey Survivor Yard</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Grey Survivor Yard from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Sundered Well</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Sundered Well from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Cracked Militia Camp</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Cracked Militia Camp from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Hollow Bread Market</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Hollow Bread Market from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Worn Stone Causeway</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Worn Stone Causeway from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Fallen Cart Road</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Fallen Cart Road from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Cold Prayer Field</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Cold Prayer Field from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Splintered Granary</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Splintered Granary from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Mourning Gatehouse</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Lords Stronghold Mourning Gatehouse from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Memory Cellar</t>
-  </si>
-  <si>
-    <t>Below Lords Stronghold Memory Cellar, the Childs thoughts split into stone, cellar dust, and old screams that invite delvers farther from daylight.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Buried Choir Mine</t>
-  </si>
-  <si>
-    <t>Below Lords Stronghold Buried Choir Mine, the Childs thoughts split into stone, cellar dust, and old screams that invite delvers farther from daylight.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Corrupted Bell Church</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Corrupted Bell Church exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Cursed Smith Anvil</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Cursed Smith Anvil exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Time Tear Obelisk</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Time Tear Obelisk exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Childs Memory Gate</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Childs Memory Gate exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Alchemy Rot Site</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Alchemy Rot Site exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Federation Wound Stronghold</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Federation Wound Stronghold exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Enemy Strength Spire</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Enemy Strength Spire exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Reality Bent Dungeon</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Reality Bent Dungeon exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Ash Wharf</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Ash Wharf keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Survivor Ferry</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Survivor Ferry keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Merchant Gate</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Merchant Gate keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Broken Crossing</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Broken Crossing keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Federation Checkpoint</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Federation Checkpoint keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Waystation Pier</t>
-  </si>
-  <si>
-    <t>Lords Stronghold Waystation Pier keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Ash-Bent Hamlet</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Ash-Bent Hamlet from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Federation Scarred Road</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Federation Scarred Road from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Starving Lantern Camp</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Starving Lantern Camp from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Drowned Merchant Post</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Drowned Merchant Post from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Broken Watch House</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Broken Watch House from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Memory-Warped Shrine</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Memory-Warped Shrine from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Famished Orchard</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Famished Orchard from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Grey Survivor Yard</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Grey Survivor Yard from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Sundered Well</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Sundered Well from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Cracked Militia Camp</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Cracked Militia Camp from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Hollow Bread Market</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Hollow Bread Market from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Worn Stone Causeway</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Worn Stone Causeway from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Fallen Cart Road</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Fallen Cart Road from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Cold Prayer Field</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Cold Prayer Field from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Splintered Granary</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Splintered Granary from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Mourning Gatehouse</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Hells Broken Anvil Mourning Gatehouse from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Memory Cellar</t>
-  </si>
-  <si>
-    <t>Below Hells Broken Anvil Memory Cellar, the Childs thoughts split into stone, cellar dust, and old screams that invite delvers farther from daylight.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Buried Choir Mine</t>
-  </si>
-  <si>
-    <t>Below Hells Broken Anvil Buried Choir Mine, the Childs thoughts split into stone, cellar dust, and old screams that invite delvers farther from daylight.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Corrupted Bell Church</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Corrupted Bell Church exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Cursed Smith Anvil</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Cursed Smith Anvil exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Time Tear Obelisk</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Time Tear Obelisk exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Childs Memory Gate</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Childs Memory Gate exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Alchemy Rot Site</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Alchemy Rot Site exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Federation Wound Stronghold</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Federation Wound Stronghold exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Enemy Strength Spire</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Enemy Strength Spire exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Reality Bent Dungeon</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Reality Bent Dungeon exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Ash Wharf</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Ash Wharf keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Survivor Ferry</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Survivor Ferry keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Merchant Gate</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Merchant Gate keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Broken Crossing</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Broken Crossing keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Federation Checkpoint</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Federation Checkpoint keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Waystation Pier</t>
-  </si>
-  <si>
-    <t>Hells Broken Anvil Waystation Pier keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
     <t>Tear in the Fabric of Time Ash-Bent Hamlet</t>
   </si>
   <si>
@@ -6188,198 +5804,6 @@
     <t>Twisted Dimensional Gate Waystation Pier keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
   </si>
   <si>
-    <t>Cave of Memories Ash-Bent Hamlet</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Ash-Bent Hamlet from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Federation Scarred Road</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Federation Scarred Road from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Starving Lantern Camp</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Starving Lantern Camp from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Drowned Merchant Post</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Drowned Merchant Post from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Broken Watch House</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Broken Watch House from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Memory-Warped Shrine</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Memory-Warped Shrine from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Famished Orchard</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Famished Orchard from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Grey Survivor Yard</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Grey Survivor Yard from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Sundered Well</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Sundered Well from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Cracked Militia Camp</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Cracked Militia Camp from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Hollow Bread Market</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Hollow Bread Market from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Worn Stone Causeway</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Worn Stone Causeway from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Fallen Cart Road</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Fallen Cart Road from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Cold Prayer Field</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Cold Prayer Field from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Splintered Granary</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Splintered Granary from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Mourning Gatehouse</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Cave of Memories Mourning Gatehouse from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Memory Cellar</t>
-  </si>
-  <si>
-    <t>Below Cave of Memories Memory Cellar, the Childs thoughts split into stone, cellar dust, and old screams that invite delvers farther from daylight.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Buried Choir Mine</t>
-  </si>
-  <si>
-    <t>Below Cave of Memories Buried Choir Mine, the Childs thoughts split into stone, cellar dust, and old screams that invite delvers farther from daylight.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Corrupted Bell Church</t>
-  </si>
-  <si>
-    <t>Cave of Memories Corrupted Bell Church exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Cursed Smith Anvil</t>
-  </si>
-  <si>
-    <t>Cave of Memories Cursed Smith Anvil exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Time Tear Obelisk</t>
-  </si>
-  <si>
-    <t>Cave of Memories Time Tear Obelisk exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Childs Memory Gate</t>
-  </si>
-  <si>
-    <t>Cave of Memories Childs Memory Gate exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Alchemy Rot Site</t>
-  </si>
-  <si>
-    <t>Cave of Memories Alchemy Rot Site exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Federation Wound Stronghold</t>
-  </si>
-  <si>
-    <t>Cave of Memories Federation Wound Stronghold exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Enemy Strength Spire</t>
-  </si>
-  <si>
-    <t>Cave of Memories Enemy Strength Spire exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Reality Bent Dungeon</t>
-  </si>
-  <si>
-    <t>Cave of Memories Reality Bent Dungeon exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Ash Wharf</t>
-  </si>
-  <si>
-    <t>Cave of Memories Ash Wharf keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Survivor Ferry</t>
-  </si>
-  <si>
-    <t>Cave of Memories Survivor Ferry keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Merchant Gate</t>
-  </si>
-  <si>
-    <t>Cave of Memories Merchant Gate keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Broken Crossing</t>
-  </si>
-  <si>
-    <t>Cave of Memories Broken Crossing keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Federation Checkpoint</t>
-  </si>
-  <si>
-    <t>Cave of Memories Federation Checkpoint keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Cave of Memories Waystation Pier</t>
-  </si>
-  <si>
-    <t>Cave of Memories Waystation Pier keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
     <t>Purgatories Dungeons Ash-Bent Hamlet</t>
   </si>
   <si>
@@ -6956,198 +6380,6 @@
     <t>Cave of Shadows Waystation Pier keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
   </si>
   <si>
-    <t>Dungeons of the twisted maiden Ash-Bent Hamlet</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Ash-Bent Hamlet from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Federation Scarred Road</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Federation Scarred Road from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Starving Lantern Camp</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Starving Lantern Camp from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Drowned Merchant Post</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Drowned Merchant Post from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Broken Watch House</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Broken Watch House from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Memory-Warped Shrine</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Memory-Warped Shrine from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Famished Orchard</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Famished Orchard from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Grey Survivor Yard</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Grey Survivor Yard from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Sundered Well</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Sundered Well from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Cracked Militia Camp</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Cracked Militia Camp from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Hollow Bread Market</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Hollow Bread Market from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Worn Stone Causeway</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Worn Stone Causeway from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Fallen Cart Road</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Fallen Cart Road from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Cold Prayer Field</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Cold Prayer Field from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Splintered Granary</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Splintered Granary from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Mourning Gatehouse</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Dungeons of the twisted maiden Mourning Gatehouse from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Memory Cellar</t>
-  </si>
-  <si>
-    <t>Below Dungeons of the twisted maiden Memory Cellar, the Childs thoughts split into stone, cellar dust, and old screams that invite delvers farther from daylight.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Buried Choir Mine</t>
-  </si>
-  <si>
-    <t>Below Dungeons of the twisted maiden Buried Choir Mine, the Childs thoughts split into stone, cellar dust, and old screams that invite delvers farther from daylight.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Corrupted Bell Church</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Corrupted Bell Church exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Cursed Smith Anvil</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Cursed Smith Anvil exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Time Tear Obelisk</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Time Tear Obelisk exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Childs Memory Gate</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Childs Memory Gate exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Alchemy Rot Site</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Alchemy Rot Site exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Federation Wound Stronghold</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Federation Wound Stronghold exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Enemy Strength Spire</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Enemy Strength Spire exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Reality Bent Dungeon</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Reality Bent Dungeon exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Ash Wharf</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Ash Wharf keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Survivor Ferry</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Survivor Ferry keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Merchant Gate</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Merchant Gate keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Broken Crossing</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Broken Crossing keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Federation Checkpoint</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Federation Checkpoint keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Waystation Pier</t>
-  </si>
-  <si>
-    <t>Dungeons of the twisted maiden Waystation Pier keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
     <t>The Old Church Ash-Bent Hamlet</t>
   </si>
   <si>
@@ -7338,198 +6570,6 @@
   </si>
   <si>
     <t>The Old Church Waystation Pier keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Ash-Bent Hamlet</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Ash-Bent Hamlet from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Federation Scarred Road</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Federation Scarred Road from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Starving Lantern Camp</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Starving Lantern Camp from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Drowned Merchant Post</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Drowned Merchant Post from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Broken Watch House</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Broken Watch House from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Memory-Warped Shrine</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Memory-Warped Shrine from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Famished Orchard</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Famished Orchard from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Grey Survivor Yard</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Grey Survivor Yard from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Sundered Well</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Sundered Well from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Cracked Militia Camp</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Cracked Militia Camp from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Hollow Bread Market</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Hollow Bread Market from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Worn Stone Causeway</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Worn Stone Causeway from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Fallen Cart Road</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Fallen Cart Road from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Cold Prayer Field</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Cold Prayer Field from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Splintered Granary</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Splintered Granary from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Mourning Gatehouse</t>
-  </si>
-  <si>
-    <t>The Childs cracking mind raises Alchemy Corrupted Church Mourning Gatehouse from hunger, mud, and Federation ruin so travelers can pretend the road still belongs to the living.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Memory Cellar</t>
-  </si>
-  <si>
-    <t>Below Alchemy Corrupted Church Memory Cellar, the Childs thoughts split into stone, cellar dust, and old screams that invite delvers farther from daylight.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Buried Choir Mine</t>
-  </si>
-  <si>
-    <t>Below Alchemy Corrupted Church Buried Choir Mine, the Childs thoughts split into stone, cellar dust, and old screams that invite delvers farther from daylight.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Corrupted Bell Church</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Corrupted Bell Church exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Cursed Smith Anvil</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Cursed Smith Anvil exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Time Tear Obelisk</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Time Tear Obelisk exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Childs Memory Gate</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Childs Memory Gate exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Alchemy Rot Site</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Alchemy Rot Site exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Federation Wound Stronghold</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Federation Wound Stronghold exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Enemy Strength Spire</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Enemy Strength Spire exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Reality Bent Dungeon</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Reality Bent Dungeon exists where the Childs failing memory tears reality around a landmark the Federation could not fully burn away.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Ash Wharf</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Ash Wharf keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Survivor Ferry</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Survivor Ferry keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Merchant Gate</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Merchant Gate keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Broken Crossing</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Broken Crossing keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Federation Checkpoint</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Federation Checkpoint keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Waystation Pier</t>
-  </si>
-  <si>
-    <t>Alchemy Corrupted Church Waystation Pier keeps a thin trade route open while sailors, refugees, and tired merchants bargain beside water darkened by war.</t>
   </si>
   <si>
     <t>Admin Reserve Regular Shelter</t>
@@ -7541,7 +6581,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="1">
     <font>
@@ -7871,11 +6911,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E1250"/>
+  <dimension ref="A1:E1090"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -23753,2348 +22793,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="1091" spans="1:5">
-      <c r="A1091" t="s">
-        <v>2187</v>
-      </c>
-      <c r="B1091" t="s">
-        <v>2188</v>
-      </c>
-      <c r="C1091" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1091">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1092" spans="1:5">
-      <c r="A1092" t="s">
-        <v>2189</v>
-      </c>
-      <c r="B1092" t="s">
-        <v>2190</v>
-      </c>
-      <c r="C1092" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1092">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1093" spans="1:5">
-      <c r="A1093" t="s">
-        <v>2191</v>
-      </c>
-      <c r="B1093" t="s">
-        <v>2192</v>
-      </c>
-      <c r="C1093" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1093">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1094" spans="1:5">
-      <c r="A1094" t="s">
-        <v>2193</v>
-      </c>
-      <c r="B1094" t="s">
-        <v>2194</v>
-      </c>
-      <c r="C1094" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1094">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1095" spans="1:5">
-      <c r="A1095" t="s">
-        <v>2195</v>
-      </c>
-      <c r="B1095" t="s">
-        <v>2196</v>
-      </c>
-      <c r="C1095" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1095">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1096" spans="1:5">
-      <c r="A1096" t="s">
-        <v>2197</v>
-      </c>
-      <c r="B1096" t="s">
-        <v>2198</v>
-      </c>
-      <c r="C1096" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1096">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1097" spans="1:5">
-      <c r="A1097" t="s">
-        <v>2199</v>
-      </c>
-      <c r="B1097" t="s">
-        <v>2200</v>
-      </c>
-      <c r="C1097" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1097">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1098" spans="1:5">
-      <c r="A1098" t="s">
-        <v>2201</v>
-      </c>
-      <c r="B1098" t="s">
-        <v>2202</v>
-      </c>
-      <c r="C1098" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1098">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1099" spans="1:5">
-      <c r="A1099" t="s">
-        <v>2203</v>
-      </c>
-      <c r="B1099" t="s">
-        <v>2204</v>
-      </c>
-      <c r="C1099" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1099">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1100" spans="1:5">
-      <c r="A1100" t="s">
-        <v>2205</v>
-      </c>
-      <c r="B1100" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C1100" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1100">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1101" spans="1:5">
-      <c r="A1101" t="s">
-        <v>2207</v>
-      </c>
-      <c r="B1101" t="s">
-        <v>2208</v>
-      </c>
-      <c r="C1101" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1101">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1102" spans="1:5">
-      <c r="A1102" t="s">
-        <v>2209</v>
-      </c>
-      <c r="B1102" t="s">
-        <v>2210</v>
-      </c>
-      <c r="C1102" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1102">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1103" spans="1:5">
-      <c r="A1103" t="s">
-        <v>2211</v>
-      </c>
-      <c r="B1103" t="s">
-        <v>2212</v>
-      </c>
-      <c r="C1103" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1103">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1104" spans="1:5">
-      <c r="A1104" t="s">
-        <v>2213</v>
-      </c>
-      <c r="B1104" t="s">
-        <v>2214</v>
-      </c>
-      <c r="C1104" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1104">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1105" spans="1:5">
-      <c r="A1105" t="s">
-        <v>2215</v>
-      </c>
-      <c r="B1105" t="s">
-        <v>2216</v>
-      </c>
-      <c r="C1105" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1105">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1106" spans="1:5">
-      <c r="A1106" t="s">
-        <v>2217</v>
-      </c>
-      <c r="B1106" t="s">
-        <v>2218</v>
-      </c>
-      <c r="C1106" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1106">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1107" spans="1:5">
-      <c r="A1107" t="s">
-        <v>2219</v>
-      </c>
-      <c r="B1107" t="s">
-        <v>2220</v>
-      </c>
-      <c r="C1107" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1107">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1108" spans="1:5">
-      <c r="A1108" t="s">
-        <v>2221</v>
-      </c>
-      <c r="B1108" t="s">
-        <v>2222</v>
-      </c>
-      <c r="C1108" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1108">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1109" spans="1:5">
-      <c r="A1109" t="s">
-        <v>2223</v>
-      </c>
-      <c r="B1109" t="s">
-        <v>2224</v>
-      </c>
-      <c r="C1109" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1109">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1110" spans="1:5">
-      <c r="A1110" t="s">
-        <v>2225</v>
-      </c>
-      <c r="B1110" t="s">
-        <v>2226</v>
-      </c>
-      <c r="C1110" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1110">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1111" spans="1:5">
-      <c r="A1111" t="s">
-        <v>2227</v>
-      </c>
-      <c r="B1111" t="s">
-        <v>2228</v>
-      </c>
-      <c r="C1111" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1111">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1112" spans="1:5">
-      <c r="A1112" t="s">
-        <v>2229</v>
-      </c>
-      <c r="B1112" t="s">
-        <v>2230</v>
-      </c>
-      <c r="C1112" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1112">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1113" spans="1:5">
-      <c r="A1113" t="s">
-        <v>2231</v>
-      </c>
-      <c r="B1113" t="s">
-        <v>2232</v>
-      </c>
-      <c r="C1113" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1113">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1114" spans="1:5">
-      <c r="A1114" t="s">
-        <v>2233</v>
-      </c>
-      <c r="B1114" t="s">
-        <v>2234</v>
-      </c>
-      <c r="C1114" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1114">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1115" spans="1:5">
-      <c r="A1115" t="s">
-        <v>2235</v>
-      </c>
-      <c r="B1115" t="s">
-        <v>2236</v>
-      </c>
-      <c r="C1115" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1115">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1116" spans="1:5">
-      <c r="A1116" t="s">
-        <v>2237</v>
-      </c>
-      <c r="B1116" t="s">
-        <v>2238</v>
-      </c>
-      <c r="C1116" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1116">
-        <v>1</v>
-      </c>
-      <c r="E1116">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1117" spans="1:5">
-      <c r="A1117" t="s">
-        <v>2239</v>
-      </c>
-      <c r="B1117" t="s">
-        <v>2240</v>
-      </c>
-      <c r="C1117" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1117">
-        <v>1</v>
-      </c>
-      <c r="E1117">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1118" spans="1:5">
-      <c r="A1118" t="s">
-        <v>2241</v>
-      </c>
-      <c r="B1118" t="s">
-        <v>2242</v>
-      </c>
-      <c r="C1118" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1118">
-        <v>1</v>
-      </c>
-      <c r="E1118">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1119" spans="1:5">
-      <c r="A1119" t="s">
-        <v>2243</v>
-      </c>
-      <c r="B1119" t="s">
-        <v>2244</v>
-      </c>
-      <c r="C1119" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1119">
-        <v>1</v>
-      </c>
-      <c r="E1119">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1120" spans="1:5">
-      <c r="A1120" t="s">
-        <v>2245</v>
-      </c>
-      <c r="B1120" t="s">
-        <v>2246</v>
-      </c>
-      <c r="C1120" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1120">
-        <v>1</v>
-      </c>
-      <c r="E1120">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1121" spans="1:5">
-      <c r="A1121" t="s">
-        <v>2247</v>
-      </c>
-      <c r="B1121" t="s">
-        <v>2248</v>
-      </c>
-      <c r="C1121" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1121">
-        <v>1</v>
-      </c>
-      <c r="E1121">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1122" spans="1:5">
-      <c r="A1122" t="s">
-        <v>2249</v>
-      </c>
-      <c r="B1122" t="s">
-        <v>2250</v>
-      </c>
-      <c r="C1122" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1122">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1123" spans="1:5">
-      <c r="A1123" t="s">
-        <v>2251</v>
-      </c>
-      <c r="B1123" t="s">
-        <v>2252</v>
-      </c>
-      <c r="C1123" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1123">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1124" spans="1:5">
-      <c r="A1124" t="s">
-        <v>2253</v>
-      </c>
-      <c r="B1124" t="s">
-        <v>2254</v>
-      </c>
-      <c r="C1124" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1124">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1125" spans="1:5">
-      <c r="A1125" t="s">
-        <v>2255</v>
-      </c>
-      <c r="B1125" t="s">
-        <v>2256</v>
-      </c>
-      <c r="C1125" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1125">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1126" spans="1:5">
-      <c r="A1126" t="s">
-        <v>2257</v>
-      </c>
-      <c r="B1126" t="s">
-        <v>2258</v>
-      </c>
-      <c r="C1126" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1126">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1127" spans="1:5">
-      <c r="A1127" t="s">
-        <v>2259</v>
-      </c>
-      <c r="B1127" t="s">
-        <v>2260</v>
-      </c>
-      <c r="C1127" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1127">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1128" spans="1:5">
-      <c r="A1128" t="s">
-        <v>2261</v>
-      </c>
-      <c r="B1128" t="s">
-        <v>2262</v>
-      </c>
-      <c r="C1128" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1128">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1129" spans="1:5">
-      <c r="A1129" t="s">
-        <v>2263</v>
-      </c>
-      <c r="B1129" t="s">
-        <v>2264</v>
-      </c>
-      <c r="C1129" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1129">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1130" spans="1:5">
-      <c r="A1130" t="s">
-        <v>2265</v>
-      </c>
-      <c r="B1130" t="s">
-        <v>2266</v>
-      </c>
-      <c r="C1130" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1130">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1131" spans="1:5">
-      <c r="A1131" t="s">
-        <v>2267</v>
-      </c>
-      <c r="B1131" t="s">
-        <v>2268</v>
-      </c>
-      <c r="C1131" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1131">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1132" spans="1:5">
-      <c r="A1132" t="s">
-        <v>2269</v>
-      </c>
-      <c r="B1132" t="s">
-        <v>2270</v>
-      </c>
-      <c r="C1132" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1132">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1133" spans="1:5">
-      <c r="A1133" t="s">
-        <v>2271</v>
-      </c>
-      <c r="B1133" t="s">
-        <v>2272</v>
-      </c>
-      <c r="C1133" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1133">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1134" spans="1:5">
-      <c r="A1134" t="s">
-        <v>2273</v>
-      </c>
-      <c r="B1134" t="s">
-        <v>2274</v>
-      </c>
-      <c r="C1134" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1134">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1135" spans="1:5">
-      <c r="A1135" t="s">
-        <v>2275</v>
-      </c>
-      <c r="B1135" t="s">
-        <v>2276</v>
-      </c>
-      <c r="C1135" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1135">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1136" spans="1:5">
-      <c r="A1136" t="s">
-        <v>2277</v>
-      </c>
-      <c r="B1136" t="s">
-        <v>2278</v>
-      </c>
-      <c r="C1136" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1136">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1137" spans="1:5">
-      <c r="A1137" t="s">
-        <v>2279</v>
-      </c>
-      <c r="B1137" t="s">
-        <v>2280</v>
-      </c>
-      <c r="C1137" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1137">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1138" spans="1:5">
-      <c r="A1138" t="s">
-        <v>2281</v>
-      </c>
-      <c r="B1138" t="s">
-        <v>2282</v>
-      </c>
-      <c r="C1138" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1138">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1139" spans="1:5">
-      <c r="A1139" t="s">
-        <v>2283</v>
-      </c>
-      <c r="B1139" t="s">
-        <v>2284</v>
-      </c>
-      <c r="C1139" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1139">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1140" spans="1:5">
-      <c r="A1140" t="s">
-        <v>2285</v>
-      </c>
-      <c r="B1140" t="s">
-        <v>2286</v>
-      </c>
-      <c r="C1140" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1140">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1141" spans="1:5">
-      <c r="A1141" t="s">
-        <v>2287</v>
-      </c>
-      <c r="B1141" t="s">
-        <v>2288</v>
-      </c>
-      <c r="C1141" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1141">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1142" spans="1:5">
-      <c r="A1142" t="s">
-        <v>2289</v>
-      </c>
-      <c r="B1142" t="s">
-        <v>2290</v>
-      </c>
-      <c r="C1142" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1142">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1143" spans="1:5">
-      <c r="A1143" t="s">
-        <v>2291</v>
-      </c>
-      <c r="B1143" t="s">
-        <v>2292</v>
-      </c>
-      <c r="C1143" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1143">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1144" spans="1:5">
-      <c r="A1144" t="s">
-        <v>2293</v>
-      </c>
-      <c r="B1144" t="s">
-        <v>2294</v>
-      </c>
-      <c r="C1144" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1144">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1145" spans="1:5">
-      <c r="A1145" t="s">
-        <v>2295</v>
-      </c>
-      <c r="B1145" t="s">
-        <v>2296</v>
-      </c>
-      <c r="C1145" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1145">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1146" spans="1:5">
-      <c r="A1146" t="s">
-        <v>2297</v>
-      </c>
-      <c r="B1146" t="s">
-        <v>2298</v>
-      </c>
-      <c r="C1146" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1146">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1147" spans="1:5">
-      <c r="A1147" t="s">
-        <v>2299</v>
-      </c>
-      <c r="B1147" t="s">
-        <v>2300</v>
-      </c>
-      <c r="C1147" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1147">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1148" spans="1:5">
-      <c r="A1148" t="s">
-        <v>2301</v>
-      </c>
-      <c r="B1148" t="s">
-        <v>2302</v>
-      </c>
-      <c r="C1148" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1148">
-        <v>1</v>
-      </c>
-      <c r="E1148">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1149" spans="1:5">
-      <c r="A1149" t="s">
-        <v>2303</v>
-      </c>
-      <c r="B1149" t="s">
-        <v>2304</v>
-      </c>
-      <c r="C1149" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1149">
-        <v>1</v>
-      </c>
-      <c r="E1149">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1150" spans="1:5">
-      <c r="A1150" t="s">
-        <v>2305</v>
-      </c>
-      <c r="B1150" t="s">
-        <v>2306</v>
-      </c>
-      <c r="C1150" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1150">
-        <v>1</v>
-      </c>
-      <c r="E1150">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1151" spans="1:5">
-      <c r="A1151" t="s">
-        <v>2307</v>
-      </c>
-      <c r="B1151" t="s">
-        <v>2308</v>
-      </c>
-      <c r="C1151" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1151">
-        <v>1</v>
-      </c>
-      <c r="E1151">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1152" spans="1:5">
-      <c r="A1152" t="s">
-        <v>2309</v>
-      </c>
-      <c r="B1152" t="s">
-        <v>2310</v>
-      </c>
-      <c r="C1152" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1152">
-        <v>1</v>
-      </c>
-      <c r="E1152">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1153" spans="1:5">
-      <c r="A1153" t="s">
-        <v>2311</v>
-      </c>
-      <c r="B1153" t="s">
-        <v>2312</v>
-      </c>
-      <c r="C1153" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1153">
-        <v>1</v>
-      </c>
-      <c r="E1153">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1154" spans="1:5">
-      <c r="A1154" t="s">
-        <v>2313</v>
-      </c>
-      <c r="B1154" t="s">
-        <v>2314</v>
-      </c>
-      <c r="C1154" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1154">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1155" spans="1:5">
-      <c r="A1155" t="s">
-        <v>2315</v>
-      </c>
-      <c r="B1155" t="s">
-        <v>2316</v>
-      </c>
-      <c r="C1155" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1155">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1156" spans="1:5">
-      <c r="A1156" t="s">
-        <v>2317</v>
-      </c>
-      <c r="B1156" t="s">
-        <v>2318</v>
-      </c>
-      <c r="C1156" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1156">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1157" spans="1:5">
-      <c r="A1157" t="s">
-        <v>2319</v>
-      </c>
-      <c r="B1157" t="s">
-        <v>2320</v>
-      </c>
-      <c r="C1157" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1157">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1158" spans="1:5">
-      <c r="A1158" t="s">
-        <v>2321</v>
-      </c>
-      <c r="B1158" t="s">
-        <v>2322</v>
-      </c>
-      <c r="C1158" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1158">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1159" spans="1:5">
-      <c r="A1159" t="s">
-        <v>2323</v>
-      </c>
-      <c r="B1159" t="s">
-        <v>2324</v>
-      </c>
-      <c r="C1159" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1159">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1160" spans="1:5">
-      <c r="A1160" t="s">
-        <v>2325</v>
-      </c>
-      <c r="B1160" t="s">
-        <v>2326</v>
-      </c>
-      <c r="C1160" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1160">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1161" spans="1:5">
-      <c r="A1161" t="s">
-        <v>2327</v>
-      </c>
-      <c r="B1161" t="s">
-        <v>2328</v>
-      </c>
-      <c r="C1161" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1161">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1162" spans="1:5">
-      <c r="A1162" t="s">
-        <v>2329</v>
-      </c>
-      <c r="B1162" t="s">
-        <v>2330</v>
-      </c>
-      <c r="C1162" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1162">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1163" spans="1:5">
-      <c r="A1163" t="s">
-        <v>2331</v>
-      </c>
-      <c r="B1163" t="s">
-        <v>2332</v>
-      </c>
-      <c r="C1163" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1163">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1164" spans="1:5">
-      <c r="A1164" t="s">
-        <v>2333</v>
-      </c>
-      <c r="B1164" t="s">
-        <v>2334</v>
-      </c>
-      <c r="C1164" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1164">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1165" spans="1:5">
-      <c r="A1165" t="s">
-        <v>2335</v>
-      </c>
-      <c r="B1165" t="s">
-        <v>2336</v>
-      </c>
-      <c r="C1165" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1165">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1166" spans="1:5">
-      <c r="A1166" t="s">
-        <v>2337</v>
-      </c>
-      <c r="B1166" t="s">
-        <v>2338</v>
-      </c>
-      <c r="C1166" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1166">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1167" spans="1:5">
-      <c r="A1167" t="s">
-        <v>2339</v>
-      </c>
-      <c r="B1167" t="s">
-        <v>2340</v>
-      </c>
-      <c r="C1167" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1167">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1168" spans="1:5">
-      <c r="A1168" t="s">
-        <v>2341</v>
-      </c>
-      <c r="B1168" t="s">
-        <v>2342</v>
-      </c>
-      <c r="C1168" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1168">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1169" spans="1:5">
-      <c r="A1169" t="s">
-        <v>2343</v>
-      </c>
-      <c r="B1169" t="s">
-        <v>2344</v>
-      </c>
-      <c r="C1169" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1169">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1170" spans="1:5">
-      <c r="A1170" t="s">
-        <v>2345</v>
-      </c>
-      <c r="B1170" t="s">
-        <v>2346</v>
-      </c>
-      <c r="C1170" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1170">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1171" spans="1:5">
-      <c r="A1171" t="s">
-        <v>2347</v>
-      </c>
-      <c r="B1171" t="s">
-        <v>2348</v>
-      </c>
-      <c r="C1171" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1171">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1172" spans="1:5">
-      <c r="A1172" t="s">
-        <v>2349</v>
-      </c>
-      <c r="B1172" t="s">
-        <v>2350</v>
-      </c>
-      <c r="C1172" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1172">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1173" spans="1:5">
-      <c r="A1173" t="s">
-        <v>2351</v>
-      </c>
-      <c r="B1173" t="s">
-        <v>2352</v>
-      </c>
-      <c r="C1173" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1173">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1174" spans="1:5">
-      <c r="A1174" t="s">
-        <v>2353</v>
-      </c>
-      <c r="B1174" t="s">
-        <v>2354</v>
-      </c>
-      <c r="C1174" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1174">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1175" spans="1:5">
-      <c r="A1175" t="s">
-        <v>2355</v>
-      </c>
-      <c r="B1175" t="s">
-        <v>2356</v>
-      </c>
-      <c r="C1175" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1175">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1176" spans="1:5">
-      <c r="A1176" t="s">
-        <v>2357</v>
-      </c>
-      <c r="B1176" t="s">
-        <v>2358</v>
-      </c>
-      <c r="C1176" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1176">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1177" spans="1:5">
-      <c r="A1177" t="s">
-        <v>2359</v>
-      </c>
-      <c r="B1177" t="s">
-        <v>2360</v>
-      </c>
-      <c r="C1177" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1177">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1178" spans="1:5">
-      <c r="A1178" t="s">
-        <v>2361</v>
-      </c>
-      <c r="B1178" t="s">
-        <v>2362</v>
-      </c>
-      <c r="C1178" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1178">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1179" spans="1:5">
-      <c r="A1179" t="s">
-        <v>2363</v>
-      </c>
-      <c r="B1179" t="s">
-        <v>2364</v>
-      </c>
-      <c r="C1179" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1179">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1180" spans="1:5">
-      <c r="A1180" t="s">
-        <v>2365</v>
-      </c>
-      <c r="B1180" t="s">
-        <v>2366</v>
-      </c>
-      <c r="C1180" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1180">
-        <v>1</v>
-      </c>
-      <c r="E1180">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1181" spans="1:5">
-      <c r="A1181" t="s">
-        <v>2367</v>
-      </c>
-      <c r="B1181" t="s">
-        <v>2368</v>
-      </c>
-      <c r="C1181" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1181">
-        <v>1</v>
-      </c>
-      <c r="E1181">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1182" spans="1:5">
-      <c r="A1182" t="s">
-        <v>2369</v>
-      </c>
-      <c r="B1182" t="s">
-        <v>2370</v>
-      </c>
-      <c r="C1182" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1182">
-        <v>1</v>
-      </c>
-      <c r="E1182">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1183" spans="1:5">
-      <c r="A1183" t="s">
-        <v>2371</v>
-      </c>
-      <c r="B1183" t="s">
-        <v>2372</v>
-      </c>
-      <c r="C1183" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1183">
-        <v>1</v>
-      </c>
-      <c r="E1183">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1184" spans="1:5">
-      <c r="A1184" t="s">
-        <v>2373</v>
-      </c>
-      <c r="B1184" t="s">
-        <v>2374</v>
-      </c>
-      <c r="C1184" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1184">
-        <v>1</v>
-      </c>
-      <c r="E1184">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1185" spans="1:5">
-      <c r="A1185" t="s">
-        <v>2375</v>
-      </c>
-      <c r="B1185" t="s">
-        <v>2376</v>
-      </c>
-      <c r="C1185" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1185">
-        <v>1</v>
-      </c>
-      <c r="E1185">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1186" spans="1:5">
-      <c r="A1186" t="s">
-        <v>2377</v>
-      </c>
-      <c r="B1186" t="s">
-        <v>2378</v>
-      </c>
-      <c r="C1186" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1186">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1187" spans="1:5">
-      <c r="A1187" t="s">
-        <v>2379</v>
-      </c>
-      <c r="B1187" t="s">
-        <v>2380</v>
-      </c>
-      <c r="C1187" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1187">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1188" spans="1:5">
-      <c r="A1188" t="s">
-        <v>2381</v>
-      </c>
-      <c r="B1188" t="s">
-        <v>2382</v>
-      </c>
-      <c r="C1188" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1188">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1189" spans="1:5">
-      <c r="A1189" t="s">
-        <v>2383</v>
-      </c>
-      <c r="B1189" t="s">
-        <v>2384</v>
-      </c>
-      <c r="C1189" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1189">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1190" spans="1:5">
-      <c r="A1190" t="s">
-        <v>2385</v>
-      </c>
-      <c r="B1190" t="s">
-        <v>2386</v>
-      </c>
-      <c r="C1190" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1190">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1191" spans="1:5">
-      <c r="A1191" t="s">
-        <v>2387</v>
-      </c>
-      <c r="B1191" t="s">
-        <v>2388</v>
-      </c>
-      <c r="C1191" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1191">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1192" spans="1:5">
-      <c r="A1192" t="s">
-        <v>2389</v>
-      </c>
-      <c r="B1192" t="s">
-        <v>2390</v>
-      </c>
-      <c r="C1192" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1192">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1193" spans="1:5">
-      <c r="A1193" t="s">
-        <v>2391</v>
-      </c>
-      <c r="B1193" t="s">
-        <v>2392</v>
-      </c>
-      <c r="C1193" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1193">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1194" spans="1:5">
-      <c r="A1194" t="s">
-        <v>2393</v>
-      </c>
-      <c r="B1194" t="s">
-        <v>2394</v>
-      </c>
-      <c r="C1194" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1194">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1195" spans="1:5">
-      <c r="A1195" t="s">
-        <v>2395</v>
-      </c>
-      <c r="B1195" t="s">
-        <v>2396</v>
-      </c>
-      <c r="C1195" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1195">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1196" spans="1:5">
-      <c r="A1196" t="s">
-        <v>2397</v>
-      </c>
-      <c r="B1196" t="s">
-        <v>2398</v>
-      </c>
-      <c r="C1196" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1196">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1197" spans="1:5">
-      <c r="A1197" t="s">
-        <v>2399</v>
-      </c>
-      <c r="B1197" t="s">
-        <v>2400</v>
-      </c>
-      <c r="C1197" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1197">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1198" spans="1:5">
-      <c r="A1198" t="s">
-        <v>2401</v>
-      </c>
-      <c r="B1198" t="s">
-        <v>2402</v>
-      </c>
-      <c r="C1198" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1198">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1199" spans="1:5">
-      <c r="A1199" t="s">
-        <v>2403</v>
-      </c>
-      <c r="B1199" t="s">
-        <v>2404</v>
-      </c>
-      <c r="C1199" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1199">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1200" spans="1:5">
-      <c r="A1200" t="s">
-        <v>2405</v>
-      </c>
-      <c r="B1200" t="s">
-        <v>2406</v>
-      </c>
-      <c r="C1200" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1200">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1201" spans="1:5">
-      <c r="A1201" t="s">
-        <v>2407</v>
-      </c>
-      <c r="B1201" t="s">
-        <v>2408</v>
-      </c>
-      <c r="C1201" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1201">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1202" spans="1:5">
-      <c r="A1202" t="s">
-        <v>2409</v>
-      </c>
-      <c r="B1202" t="s">
-        <v>2410</v>
-      </c>
-      <c r="C1202" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1202">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1203" spans="1:5">
-      <c r="A1203" t="s">
-        <v>2411</v>
-      </c>
-      <c r="B1203" t="s">
-        <v>2412</v>
-      </c>
-      <c r="C1203" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1203">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1204" spans="1:5">
-      <c r="A1204" t="s">
-        <v>2413</v>
-      </c>
-      <c r="B1204" t="s">
-        <v>2414</v>
-      </c>
-      <c r="C1204" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1204">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1205" spans="1:5">
-      <c r="A1205" t="s">
-        <v>2415</v>
-      </c>
-      <c r="B1205" t="s">
-        <v>2416</v>
-      </c>
-      <c r="C1205" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1205">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1206" spans="1:5">
-      <c r="A1206" t="s">
-        <v>2417</v>
-      </c>
-      <c r="B1206" t="s">
-        <v>2418</v>
-      </c>
-      <c r="C1206" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1206">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1207" spans="1:5">
-      <c r="A1207" t="s">
-        <v>2419</v>
-      </c>
-      <c r="B1207" t="s">
-        <v>2420</v>
-      </c>
-      <c r="C1207" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1207">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1208" spans="1:5">
-      <c r="A1208" t="s">
-        <v>2421</v>
-      </c>
-      <c r="B1208" t="s">
-        <v>2422</v>
-      </c>
-      <c r="C1208" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1208">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1209" spans="1:5">
-      <c r="A1209" t="s">
-        <v>2423</v>
-      </c>
-      <c r="B1209" t="s">
-        <v>2424</v>
-      </c>
-      <c r="C1209" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1209">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1210" spans="1:5">
-      <c r="A1210" t="s">
-        <v>2425</v>
-      </c>
-      <c r="B1210" t="s">
-        <v>2426</v>
-      </c>
-      <c r="C1210" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1210">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1211" spans="1:5">
-      <c r="A1211" t="s">
-        <v>2427</v>
-      </c>
-      <c r="B1211" t="s">
-        <v>2428</v>
-      </c>
-      <c r="C1211" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1211">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1212" spans="1:5">
-      <c r="A1212" t="s">
-        <v>2429</v>
-      </c>
-      <c r="B1212" t="s">
-        <v>2430</v>
-      </c>
-      <c r="C1212" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1212">
-        <v>1</v>
-      </c>
-      <c r="E1212">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1213" spans="1:5">
-      <c r="A1213" t="s">
-        <v>2431</v>
-      </c>
-      <c r="B1213" t="s">
-        <v>2432</v>
-      </c>
-      <c r="C1213" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1213">
-        <v>1</v>
-      </c>
-      <c r="E1213">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1214" spans="1:5">
-      <c r="A1214" t="s">
-        <v>2433</v>
-      </c>
-      <c r="B1214" t="s">
-        <v>2434</v>
-      </c>
-      <c r="C1214" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1214">
-        <v>1</v>
-      </c>
-      <c r="E1214">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1215" spans="1:5">
-      <c r="A1215" t="s">
-        <v>2435</v>
-      </c>
-      <c r="B1215" t="s">
-        <v>2436</v>
-      </c>
-      <c r="C1215" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1215">
-        <v>1</v>
-      </c>
-      <c r="E1215">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1216" spans="1:5">
-      <c r="A1216" t="s">
-        <v>2437</v>
-      </c>
-      <c r="B1216" t="s">
-        <v>2438</v>
-      </c>
-      <c r="C1216" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1216">
-        <v>1</v>
-      </c>
-      <c r="E1216">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1217" spans="1:5">
-      <c r="A1217" t="s">
-        <v>2439</v>
-      </c>
-      <c r="B1217" t="s">
-        <v>2440</v>
-      </c>
-      <c r="C1217" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1217">
-        <v>1</v>
-      </c>
-      <c r="E1217">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1218" spans="1:5">
-      <c r="A1218" t="s">
-        <v>2441</v>
-      </c>
-      <c r="B1218" t="s">
-        <v>2442</v>
-      </c>
-      <c r="C1218" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1218">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1219" spans="1:5">
-      <c r="A1219" t="s">
-        <v>2443</v>
-      </c>
-      <c r="B1219" t="s">
-        <v>2444</v>
-      </c>
-      <c r="C1219" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1219">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1220" spans="1:5">
-      <c r="A1220" t="s">
-        <v>2445</v>
-      </c>
-      <c r="B1220" t="s">
-        <v>2446</v>
-      </c>
-      <c r="C1220" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1220">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1221" spans="1:5">
-      <c r="A1221" t="s">
-        <v>2447</v>
-      </c>
-      <c r="B1221" t="s">
-        <v>2448</v>
-      </c>
-      <c r="C1221" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1221">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1222" spans="1:5">
-      <c r="A1222" t="s">
-        <v>2449</v>
-      </c>
-      <c r="B1222" t="s">
-        <v>2450</v>
-      </c>
-      <c r="C1222" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1222">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1223" spans="1:5">
-      <c r="A1223" t="s">
-        <v>2451</v>
-      </c>
-      <c r="B1223" t="s">
-        <v>2452</v>
-      </c>
-      <c r="C1223" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1223">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1224" spans="1:5">
-      <c r="A1224" t="s">
-        <v>2453</v>
-      </c>
-      <c r="B1224" t="s">
-        <v>2454</v>
-      </c>
-      <c r="C1224" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1224">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1225" spans="1:5">
-      <c r="A1225" t="s">
-        <v>2455</v>
-      </c>
-      <c r="B1225" t="s">
-        <v>2456</v>
-      </c>
-      <c r="C1225" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1225">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1226" spans="1:5">
-      <c r="A1226" t="s">
-        <v>2457</v>
-      </c>
-      <c r="B1226" t="s">
-        <v>2458</v>
-      </c>
-      <c r="C1226" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1226">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1227" spans="1:5">
-      <c r="A1227" t="s">
-        <v>2459</v>
-      </c>
-      <c r="B1227" t="s">
-        <v>2460</v>
-      </c>
-      <c r="C1227" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1227">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1228" spans="1:5">
-      <c r="A1228" t="s">
-        <v>2461</v>
-      </c>
-      <c r="B1228" t="s">
-        <v>2462</v>
-      </c>
-      <c r="C1228" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1228">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1229" spans="1:5">
-      <c r="A1229" t="s">
-        <v>2463</v>
-      </c>
-      <c r="B1229" t="s">
-        <v>2464</v>
-      </c>
-      <c r="C1229" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1229">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1230" spans="1:5">
-      <c r="A1230" t="s">
-        <v>2465</v>
-      </c>
-      <c r="B1230" t="s">
-        <v>2466</v>
-      </c>
-      <c r="C1230" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1230">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1231" spans="1:5">
-      <c r="A1231" t="s">
-        <v>2467</v>
-      </c>
-      <c r="B1231" t="s">
-        <v>2468</v>
-      </c>
-      <c r="C1231" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1231">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1232" spans="1:5">
-      <c r="A1232" t="s">
-        <v>2469</v>
-      </c>
-      <c r="B1232" t="s">
-        <v>2470</v>
-      </c>
-      <c r="C1232" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1232">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1233" spans="1:5">
-      <c r="A1233" t="s">
-        <v>2471</v>
-      </c>
-      <c r="B1233" t="s">
-        <v>2472</v>
-      </c>
-      <c r="C1233" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1233">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1234" spans="1:5">
-      <c r="A1234" t="s">
-        <v>2473</v>
-      </c>
-      <c r="B1234" t="s">
-        <v>2474</v>
-      </c>
-      <c r="C1234" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1234">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1235" spans="1:5">
-      <c r="A1235" t="s">
-        <v>2475</v>
-      </c>
-      <c r="B1235" t="s">
-        <v>2476</v>
-      </c>
-      <c r="C1235" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1235">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1236" spans="1:5">
-      <c r="A1236" t="s">
-        <v>2477</v>
-      </c>
-      <c r="B1236" t="s">
-        <v>2478</v>
-      </c>
-      <c r="C1236" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1236">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1237" spans="1:5">
-      <c r="A1237" t="s">
-        <v>2479</v>
-      </c>
-      <c r="B1237" t="s">
-        <v>2480</v>
-      </c>
-      <c r="C1237" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1237">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1238" spans="1:5">
-      <c r="A1238" t="s">
-        <v>2481</v>
-      </c>
-      <c r="B1238" t="s">
-        <v>2482</v>
-      </c>
-      <c r="C1238" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1238">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1239" spans="1:5">
-      <c r="A1239" t="s">
-        <v>2483</v>
-      </c>
-      <c r="B1239" t="s">
-        <v>2484</v>
-      </c>
-      <c r="C1239" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1239">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1240" spans="1:5">
-      <c r="A1240" t="s">
-        <v>2485</v>
-      </c>
-      <c r="B1240" t="s">
-        <v>2486</v>
-      </c>
-      <c r="C1240" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1240">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1241" spans="1:5">
-      <c r="A1241" t="s">
-        <v>2487</v>
-      </c>
-      <c r="B1241" t="s">
-        <v>2488</v>
-      </c>
-      <c r="C1241" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1241">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1242" spans="1:5">
-      <c r="A1242" t="s">
-        <v>2489</v>
-      </c>
-      <c r="B1242" t="s">
-        <v>2490</v>
-      </c>
-      <c r="C1242" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1242">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1243" spans="1:5">
-      <c r="A1243" t="s">
-        <v>2491</v>
-      </c>
-      <c r="B1243" t="s">
-        <v>2492</v>
-      </c>
-      <c r="C1243" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1243">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1244" spans="1:5">
-      <c r="A1244" t="s">
-        <v>2493</v>
-      </c>
-      <c r="B1244" t="s">
-        <v>2494</v>
-      </c>
-      <c r="C1244" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1244">
-        <v>1</v>
-      </c>
-      <c r="E1244">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1245" spans="1:5">
-      <c r="A1245" t="s">
-        <v>2495</v>
-      </c>
-      <c r="B1245" t="s">
-        <v>2496</v>
-      </c>
-      <c r="C1245" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1245">
-        <v>1</v>
-      </c>
-      <c r="E1245">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1246" spans="1:5">
-      <c r="A1246" t="s">
-        <v>2497</v>
-      </c>
-      <c r="B1246" t="s">
-        <v>2498</v>
-      </c>
-      <c r="C1246" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1246">
-        <v>1</v>
-      </c>
-      <c r="E1246">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1247" spans="1:5">
-      <c r="A1247" t="s">
-        <v>2499</v>
-      </c>
-      <c r="B1247" t="s">
-        <v>2500</v>
-      </c>
-      <c r="C1247" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1247">
-        <v>1</v>
-      </c>
-      <c r="E1247">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1248" spans="1:5">
-      <c r="A1248" t="s">
-        <v>2501</v>
-      </c>
-      <c r="B1248" t="s">
-        <v>2502</v>
-      </c>
-      <c r="C1248" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1248">
-        <v>1</v>
-      </c>
-      <c r="E1248">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1249" spans="1:5">
-      <c r="A1249" t="s">
-        <v>2503</v>
-      </c>
-      <c r="B1249" t="s">
-        <v>2504</v>
-      </c>
-      <c r="C1249" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1249">
-        <v>1</v>
-      </c>
-      <c r="E1249">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1250" spans="1:5">
-      <c r="A1250" t="s">
-        <v>2505</v>
-      </c>
-      <c r="B1250" t="s">
-        <v>2506</v>
-      </c>
-      <c r="C1250" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1250">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>